<commit_message>
Even more on accruals excel files and mappings
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/CATE.ST.xlsx
+++ b/data/stx_xlsx/CATE.ST.xlsx
@@ -9525,7 +9525,9 @@
       <c r="R25" s="16">
         <v>82.99</v>
       </c>
-      <c r="S25" s="20"/>
+      <c r="S25" s="16">
+        <v>40.15</v>
+      </c>
       <c r="T25" s="16">
         <v>29.82</v>
       </c>
@@ -10116,13 +10118,34 @@
         <v>1.04</v>
       </c>
       <c r="O39" s="20"/>
-      <c r="P39" s="20"/>
-      <c r="Q39" s="20"/>
-      <c r="R39" s="20"/>
-      <c r="S39" s="20"/>
-      <c r="T39" s="20"/>
-      <c r="U39" s="20"/>
-      <c r="V39" s="20"/>
+      <c r="P39" s="16">
+        <f t="shared" ref="P39:V39" si="1">SUM(P40:P41)</f>
+        <v>0.01</v>
+      </c>
+      <c r="Q39" s="16">
+        <f t="shared" si="1"/>
+        <v>1.18</v>
+      </c>
+      <c r="R39" s="16">
+        <f t="shared" si="1"/>
+        <v>1.58</v>
+      </c>
+      <c r="S39" s="16">
+        <f t="shared" si="1"/>
+        <v>2.23</v>
+      </c>
+      <c r="T39" s="16">
+        <f t="shared" si="1"/>
+        <v>2.92</v>
+      </c>
+      <c r="U39" s="16">
+        <f t="shared" si="1"/>
+        <v>3.76</v>
+      </c>
+      <c r="V39" s="16">
+        <f t="shared" si="1"/>
+        <v>1.79</v>
+      </c>
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">

</xml_diff>